<commit_message>
Complete Phase 2 - all routins , stories and modules in Simulator app are ready , and also add an example for a log in the sim_log folder
</commit_message>
<xml_diff>
--- a/routines/David.xlsx
+++ b/routines/David.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\itay3\Desktop\Projects\EnsoSphere_IoT_Project\routines\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{116F15E1-F4F2-4C19-9592-9E9F95036267}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A93AC38-FB4B-479A-92D9-CFD6C1C716A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1515" windowWidth="21600" windowHeight="13830" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="13830" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="New Text Document" sheetId="1" r:id="rId1"/>
@@ -1167,10 +1167,10 @@
         <v>16</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C5" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D5" t="s">
         <v>8</v>

</xml_diff>